<commit_message>
Nota en el resumen del xlsx de auditoria (recalculo no disponible en el contenedor)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FYWyG35uyB8TYJDn12HUYM
</commit_message>
<xml_diff>
--- a/josh_auditoria_manual_2025.xlsx
+++ b/josh_auditoria_manual_2025.xlsx
@@ -16,10 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.00000"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -140,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,9 +157,9 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -172,6 +171,8 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -724,7 +725,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="21" t="n">
         <v>45658</v>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -754,7 +755,7 @@
       <c r="N7" s="12" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="22" t="n">
         <v>45659</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -784,7 +785,7 @@
       <c r="N8" s="17" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n">
+      <c r="A9" s="22" t="n">
         <v>45660</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -824,7 +825,7 @@
       <c r="N9" s="17" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="n">
+      <c r="A10" s="22" t="n">
         <v>45663</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -874,7 +875,7 @@
       <c r="N10" s="17" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="n">
+      <c r="A11" s="22" t="n">
         <v>45664</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -924,7 +925,7 @@
       <c r="N11" s="17" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="n">
+      <c r="A12" s="22" t="n">
         <v>45665</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -964,7 +965,7 @@
       <c r="N12" s="17" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="n">
+      <c r="A13" s="22" t="n">
         <v>45666</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -1014,7 +1015,7 @@
       <c r="N13" s="17" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="n">
+      <c r="A14" s="22" t="n">
         <v>45667</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -1064,7 +1065,7 @@
       <c r="N14" s="17" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="n">
+      <c r="A15" s="22" t="n">
         <v>45670</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -1104,7 +1105,7 @@
       <c r="N15" s="17" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="n">
+      <c r="A16" s="22" t="n">
         <v>45671</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -1134,7 +1135,7 @@
       <c r="N16" s="17" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="n">
+      <c r="A17" s="22" t="n">
         <v>45672</v>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -1184,7 +1185,7 @@
       <c r="N17" s="17" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="n">
+      <c r="A18" s="22" t="n">
         <v>45673</v>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -1234,7 +1235,7 @@
       <c r="N18" s="17" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="n">
+      <c r="A19" s="22" t="n">
         <v>45674</v>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -1284,7 +1285,7 @@
       <c r="N19" s="17" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="n">
+      <c r="A20" s="22" t="n">
         <v>45677</v>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -1324,7 +1325,7 @@
       <c r="N20" s="17" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="n">
+      <c r="A21" s="22" t="n">
         <v>45678</v>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -1374,7 +1375,7 @@
       <c r="N21" s="17" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="n">
+      <c r="A22" s="22" t="n">
         <v>45679</v>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -1414,7 +1415,7 @@
       <c r="N22" s="17" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="n">
+      <c r="A23" s="22" t="n">
         <v>45680</v>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -1464,7 +1465,7 @@
       <c r="N23" s="17" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="n">
+      <c r="A24" s="22" t="n">
         <v>45681</v>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -1504,7 +1505,7 @@
       <c r="N24" s="17" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n">
+      <c r="A25" s="22" t="n">
         <v>45684</v>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -1554,7 +1555,7 @@
       <c r="N25" s="17" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="n">
+      <c r="A26" s="22" t="n">
         <v>45685</v>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -1594,7 +1595,7 @@
       <c r="N26" s="17" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="n">
+      <c r="A27" s="22" t="n">
         <v>45686</v>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -1644,7 +1645,7 @@
       <c r="N27" s="17" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="n">
+      <c r="A28" s="22" t="n">
         <v>45687</v>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -1694,7 +1695,7 @@
       <c r="N28" s="17" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="n">
+      <c r="A29" s="22" t="n">
         <v>45688</v>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -1744,7 +1745,7 @@
       <c r="N29" s="17" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="n">
+      <c r="A30" s="22" t="n">
         <v>45691</v>
       </c>
       <c r="B30" s="14" t="inlineStr">
@@ -1784,7 +1785,7 @@
       <c r="N30" s="17" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="n">
+      <c r="A31" s="22" t="n">
         <v>45692</v>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -1834,7 +1835,7 @@
       <c r="N31" s="17" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="n">
+      <c r="A32" s="22" t="n">
         <v>45693</v>
       </c>
       <c r="B32" s="14" t="inlineStr">
@@ -1874,7 +1875,7 @@
       <c r="N32" s="17" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="n">
+      <c r="A33" s="22" t="n">
         <v>45694</v>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -1914,7 +1915,7 @@
       <c r="N33" s="17" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="n">
+      <c r="A34" s="22" t="n">
         <v>45695</v>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -1964,7 +1965,7 @@
       <c r="N34" s="17" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="n">
+      <c r="A35" s="22" t="n">
         <v>45698</v>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -2014,7 +2015,7 @@
       <c r="N35" s="17" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="n">
+      <c r="A36" s="22" t="n">
         <v>45699</v>
       </c>
       <c r="B36" s="14" t="inlineStr">
@@ -2054,7 +2055,7 @@
       <c r="N36" s="17" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="n">
+      <c r="A37" s="22" t="n">
         <v>45700</v>
       </c>
       <c r="B37" s="14" t="inlineStr">
@@ -2094,7 +2095,7 @@
       <c r="N37" s="17" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="n">
+      <c r="A38" s="22" t="n">
         <v>45701</v>
       </c>
       <c r="B38" s="14" t="inlineStr">
@@ -2144,7 +2145,7 @@
       <c r="N38" s="17" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="n">
+      <c r="A39" s="22" t="n">
         <v>45702</v>
       </c>
       <c r="B39" s="14" t="inlineStr">
@@ -2184,7 +2185,7 @@
       <c r="N39" s="17" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="n">
+      <c r="A40" s="22" t="n">
         <v>45705</v>
       </c>
       <c r="B40" s="14" t="inlineStr">
@@ -2234,7 +2235,7 @@
       <c r="N40" s="17" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="n">
+      <c r="A41" s="22" t="n">
         <v>45706</v>
       </c>
       <c r="B41" s="14" t="inlineStr">
@@ -2274,7 +2275,7 @@
       <c r="N41" s="17" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="n">
+      <c r="A42" s="22" t="n">
         <v>45707</v>
       </c>
       <c r="B42" s="14" t="inlineStr">
@@ -2324,7 +2325,7 @@
       <c r="N42" s="17" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="13" t="n">
+      <c r="A43" s="22" t="n">
         <v>45708</v>
       </c>
       <c r="B43" s="14" t="inlineStr">
@@ -2364,7 +2365,7 @@
       <c r="N43" s="17" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="13" t="n">
+      <c r="A44" s="22" t="n">
         <v>45709</v>
       </c>
       <c r="B44" s="14" t="inlineStr">
@@ -2404,7 +2405,7 @@
       <c r="N44" s="17" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="n">
+      <c r="A45" s="22" t="n">
         <v>45712</v>
       </c>
       <c r="B45" s="14" t="inlineStr">
@@ -2444,7 +2445,7 @@
       <c r="N45" s="17" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="13" t="n">
+      <c r="A46" s="22" t="n">
         <v>45713</v>
       </c>
       <c r="B46" s="14" t="inlineStr">
@@ -2484,7 +2485,7 @@
       <c r="N46" s="17" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="n">
+      <c r="A47" s="22" t="n">
         <v>45714</v>
       </c>
       <c r="B47" s="14" t="inlineStr">
@@ -2524,7 +2525,7 @@
       <c r="N47" s="17" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="n">
+      <c r="A48" s="22" t="n">
         <v>45715</v>
       </c>
       <c r="B48" s="14" t="inlineStr">
@@ -2564,7 +2565,7 @@
       <c r="N48" s="17" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="n">
+      <c r="A49" s="22" t="n">
         <v>45716</v>
       </c>
       <c r="B49" s="14" t="inlineStr">
@@ -2614,7 +2615,7 @@
       <c r="N49" s="17" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="n">
+      <c r="A50" s="22" t="n">
         <v>45719</v>
       </c>
       <c r="B50" s="14" t="inlineStr">
@@ -2664,7 +2665,7 @@
       <c r="N50" s="17" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="13" t="n">
+      <c r="A51" s="22" t="n">
         <v>45720</v>
       </c>
       <c r="B51" s="14" t="inlineStr">
@@ -2714,7 +2715,7 @@
       <c r="N51" s="17" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="n">
+      <c r="A52" s="22" t="n">
         <v>45721</v>
       </c>
       <c r="B52" s="14" t="inlineStr">
@@ -2764,7 +2765,7 @@
       <c r="N52" s="17" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="n">
+      <c r="A53" s="22" t="n">
         <v>45722</v>
       </c>
       <c r="B53" s="14" t="inlineStr">
@@ -2814,7 +2815,7 @@
       <c r="N53" s="17" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="13" t="n">
+      <c r="A54" s="22" t="n">
         <v>45723</v>
       </c>
       <c r="B54" s="14" t="inlineStr">
@@ -2864,7 +2865,7 @@
       <c r="N54" s="17" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="13" t="n">
+      <c r="A55" s="22" t="n">
         <v>45726</v>
       </c>
       <c r="B55" s="14" t="inlineStr">
@@ -2914,7 +2915,7 @@
       <c r="N55" s="17" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="13" t="n">
+      <c r="A56" s="22" t="n">
         <v>45727</v>
       </c>
       <c r="B56" s="14" t="inlineStr">
@@ -2964,7 +2965,7 @@
       <c r="N56" s="17" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="13" t="n">
+      <c r="A57" s="22" t="n">
         <v>45728</v>
       </c>
       <c r="B57" s="14" t="inlineStr">
@@ -3014,7 +3015,7 @@
       <c r="N57" s="17" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="13" t="n">
+      <c r="A58" s="22" t="n">
         <v>45729</v>
       </c>
       <c r="B58" s="14" t="inlineStr">
@@ -3064,7 +3065,7 @@
       <c r="N58" s="17" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="13" t="n">
+      <c r="A59" s="22" t="n">
         <v>45730</v>
       </c>
       <c r="B59" s="14" t="inlineStr">
@@ -3114,7 +3115,7 @@
       <c r="N59" s="17" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="13" t="n">
+      <c r="A60" s="22" t="n">
         <v>45733</v>
       </c>
       <c r="B60" s="14" t="inlineStr">
@@ -3164,7 +3165,7 @@
       <c r="N60" s="17" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="13" t="n">
+      <c r="A61" s="22" t="n">
         <v>45734</v>
       </c>
       <c r="B61" s="14" t="inlineStr">
@@ -3204,7 +3205,7 @@
       <c r="N61" s="17" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="13" t="n">
+      <c r="A62" s="22" t="n">
         <v>45735</v>
       </c>
       <c r="B62" s="14" t="inlineStr">
@@ -3254,7 +3255,7 @@
       <c r="N62" s="17" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="13" t="n">
+      <c r="A63" s="22" t="n">
         <v>45736</v>
       </c>
       <c r="B63" s="14" t="inlineStr">
@@ -3294,7 +3295,7 @@
       <c r="N63" s="17" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="13" t="n">
+      <c r="A64" s="22" t="n">
         <v>45737</v>
       </c>
       <c r="B64" s="14" t="inlineStr">
@@ -3344,7 +3345,7 @@
       <c r="N64" s="17" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="13" t="n">
+      <c r="A65" s="22" t="n">
         <v>45740</v>
       </c>
       <c r="B65" s="14" t="inlineStr">
@@ -3394,7 +3395,7 @@
       <c r="N65" s="17" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="13" t="n">
+      <c r="A66" s="22" t="n">
         <v>45741</v>
       </c>
       <c r="B66" s="14" t="inlineStr">
@@ -3444,7 +3445,7 @@
       <c r="N66" s="17" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="13" t="n">
+      <c r="A67" s="22" t="n">
         <v>45742</v>
       </c>
       <c r="B67" s="14" t="inlineStr">
@@ -3494,7 +3495,7 @@
       <c r="N67" s="17" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="13" t="n">
+      <c r="A68" s="22" t="n">
         <v>45743</v>
       </c>
       <c r="B68" s="14" t="inlineStr">
@@ -3524,7 +3525,7 @@
       <c r="N68" s="17" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="13" t="n">
+      <c r="A69" s="22" t="n">
         <v>45744</v>
       </c>
       <c r="B69" s="14" t="inlineStr">
@@ -3574,7 +3575,7 @@
       <c r="N69" s="17" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="13" t="n">
+      <c r="A70" s="22" t="n">
         <v>45747</v>
       </c>
       <c r="B70" s="14" t="inlineStr">
@@ -3624,7 +3625,7 @@
       <c r="N70" s="17" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="13" t="n">
+      <c r="A71" s="22" t="n">
         <v>45748</v>
       </c>
       <c r="B71" s="14" t="inlineStr">
@@ -3664,7 +3665,7 @@
       <c r="N71" s="17" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="13" t="n">
+      <c r="A72" s="22" t="n">
         <v>45749</v>
       </c>
       <c r="B72" s="14" t="inlineStr">
@@ -3714,7 +3715,7 @@
       <c r="N72" s="17" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="13" t="n">
+      <c r="A73" s="22" t="n">
         <v>45750</v>
       </c>
       <c r="B73" s="14" t="inlineStr">
@@ -3754,7 +3755,7 @@
       <c r="N73" s="17" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="13" t="n">
+      <c r="A74" s="22" t="n">
         <v>45751</v>
       </c>
       <c r="B74" s="14" t="inlineStr">
@@ -3804,7 +3805,7 @@
       <c r="N74" s="17" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="13" t="n">
+      <c r="A75" s="22" t="n">
         <v>45754</v>
       </c>
       <c r="B75" s="14" t="inlineStr">
@@ -3854,7 +3855,7 @@
       <c r="N75" s="17" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="13" t="n">
+      <c r="A76" s="22" t="n">
         <v>45755</v>
       </c>
       <c r="B76" s="14" t="inlineStr">
@@ -3904,7 +3905,7 @@
       <c r="N76" s="17" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="13" t="n">
+      <c r="A77" s="22" t="n">
         <v>45756</v>
       </c>
       <c r="B77" s="14" t="inlineStr">
@@ -3954,7 +3955,7 @@
       <c r="N77" s="17" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="13" t="n">
+      <c r="A78" s="22" t="n">
         <v>45757</v>
       </c>
       <c r="B78" s="14" t="inlineStr">
@@ -3994,7 +3995,7 @@
       <c r="N78" s="17" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="13" t="n">
+      <c r="A79" s="22" t="n">
         <v>45758</v>
       </c>
       <c r="B79" s="14" t="inlineStr">
@@ -4034,7 +4035,7 @@
       <c r="N79" s="17" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="13" t="n">
+      <c r="A80" s="22" t="n">
         <v>45761</v>
       </c>
       <c r="B80" s="14" t="inlineStr">
@@ -4084,7 +4085,7 @@
       <c r="N80" s="17" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="13" t="n">
+      <c r="A81" s="22" t="n">
         <v>45762</v>
       </c>
       <c r="B81" s="14" t="inlineStr">
@@ -4134,7 +4135,7 @@
       <c r="N81" s="17" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="13" t="n">
+      <c r="A82" s="22" t="n">
         <v>45763</v>
       </c>
       <c r="B82" s="14" t="inlineStr">
@@ -4184,7 +4185,7 @@
       <c r="N82" s="17" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="13" t="n">
+      <c r="A83" s="22" t="n">
         <v>45764</v>
       </c>
       <c r="B83" s="14" t="inlineStr">
@@ -4234,7 +4235,7 @@
       <c r="N83" s="17" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="13" t="n">
+      <c r="A84" s="22" t="n">
         <v>45765</v>
       </c>
       <c r="B84" s="14" t="inlineStr">
@@ -4284,7 +4285,7 @@
       <c r="N84" s="17" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="13" t="n">
+      <c r="A85" s="22" t="n">
         <v>45768</v>
       </c>
       <c r="B85" s="14" t="inlineStr">
@@ -4334,7 +4335,7 @@
       <c r="N85" s="17" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="13" t="n">
+      <c r="A86" s="22" t="n">
         <v>45769</v>
       </c>
       <c r="B86" s="14" t="inlineStr">
@@ -4374,7 +4375,7 @@
       <c r="N86" s="17" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="13" t="n">
+      <c r="A87" s="22" t="n">
         <v>45770</v>
       </c>
       <c r="B87" s="14" t="inlineStr">
@@ -4414,7 +4415,7 @@
       <c r="N87" s="17" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="13" t="n">
+      <c r="A88" s="22" t="n">
         <v>45771</v>
       </c>
       <c r="B88" s="14" t="inlineStr">
@@ -4454,7 +4455,7 @@
       <c r="N88" s="17" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="13" t="n">
+      <c r="A89" s="22" t="n">
         <v>45772</v>
       </c>
       <c r="B89" s="14" t="inlineStr">
@@ -4504,7 +4505,7 @@
       <c r="N89" s="17" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="13" t="n">
+      <c r="A90" s="22" t="n">
         <v>45775</v>
       </c>
       <c r="B90" s="14" t="inlineStr">
@@ -4554,7 +4555,7 @@
       <c r="N90" s="17" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="13" t="n">
+      <c r="A91" s="22" t="n">
         <v>45776</v>
       </c>
       <c r="B91" s="14" t="inlineStr">
@@ -4604,7 +4605,7 @@
       <c r="N91" s="17" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="13" t="n">
+      <c r="A92" s="22" t="n">
         <v>45777</v>
       </c>
       <c r="B92" s="14" t="inlineStr">
@@ -4634,7 +4635,7 @@
       <c r="N92" s="17" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="13" t="n">
+      <c r="A93" s="22" t="n">
         <v>45778</v>
       </c>
       <c r="B93" s="14" t="inlineStr">
@@ -4684,7 +4685,7 @@
       <c r="N93" s="17" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="13" t="n">
+      <c r="A94" s="22" t="n">
         <v>45779</v>
       </c>
       <c r="B94" s="14" t="inlineStr">
@@ -4734,7 +4735,7 @@
       <c r="N94" s="17" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="13" t="n">
+      <c r="A95" s="22" t="n">
         <v>45782</v>
       </c>
       <c r="B95" s="14" t="inlineStr">
@@ -4784,7 +4785,7 @@
       <c r="N95" s="17" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="13" t="n">
+      <c r="A96" s="22" t="n">
         <v>45783</v>
       </c>
       <c r="B96" s="14" t="inlineStr">
@@ -4834,7 +4835,7 @@
       <c r="N96" s="17" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="13" t="n">
+      <c r="A97" s="22" t="n">
         <v>45784</v>
       </c>
       <c r="B97" s="14" t="inlineStr">
@@ -4864,7 +4865,7 @@
       <c r="N97" s="17" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="13" t="n">
+      <c r="A98" s="22" t="n">
         <v>45785</v>
       </c>
       <c r="B98" s="14" t="inlineStr">
@@ -4914,7 +4915,7 @@
       <c r="N98" s="17" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="13" t="n">
+      <c r="A99" s="22" t="n">
         <v>45786</v>
       </c>
       <c r="B99" s="14" t="inlineStr">
@@ -4964,7 +4965,7 @@
       <c r="N99" s="17" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="13" t="n">
+      <c r="A100" s="22" t="n">
         <v>45789</v>
       </c>
       <c r="B100" s="14" t="inlineStr">
@@ -5004,7 +5005,7 @@
       <c r="N100" s="17" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="13" t="n">
+      <c r="A101" s="22" t="n">
         <v>45790</v>
       </c>
       <c r="B101" s="14" t="inlineStr">
@@ -5054,7 +5055,7 @@
       <c r="N101" s="17" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="13" t="n">
+      <c r="A102" s="22" t="n">
         <v>45791</v>
       </c>
       <c r="B102" s="14" t="inlineStr">
@@ -5104,7 +5105,7 @@
       <c r="N102" s="17" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="13" t="n">
+      <c r="A103" s="22" t="n">
         <v>45792</v>
       </c>
       <c r="B103" s="14" t="inlineStr">
@@ -5144,7 +5145,7 @@
       <c r="N103" s="17" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="13" t="n">
+      <c r="A104" s="22" t="n">
         <v>45793</v>
       </c>
       <c r="B104" s="14" t="inlineStr">
@@ -5194,7 +5195,7 @@
       <c r="N104" s="17" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="13" t="n">
+      <c r="A105" s="22" t="n">
         <v>45796</v>
       </c>
       <c r="B105" s="14" t="inlineStr">
@@ -5234,7 +5235,7 @@
       <c r="N105" s="17" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="13" t="n">
+      <c r="A106" s="22" t="n">
         <v>45797</v>
       </c>
       <c r="B106" s="14" t="inlineStr">
@@ -5284,7 +5285,7 @@
       <c r="N106" s="17" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="13" t="n">
+      <c r="A107" s="22" t="n">
         <v>45798</v>
       </c>
       <c r="B107" s="14" t="inlineStr">
@@ -5324,7 +5325,7 @@
       <c r="N107" s="17" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="13" t="n">
+      <c r="A108" s="22" t="n">
         <v>45799</v>
       </c>
       <c r="B108" s="14" t="inlineStr">
@@ -5374,7 +5375,7 @@
       <c r="N108" s="17" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="13" t="n">
+      <c r="A109" s="22" t="n">
         <v>45800</v>
       </c>
       <c r="B109" s="14" t="inlineStr">
@@ -5424,7 +5425,7 @@
       <c r="N109" s="17" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="13" t="n">
+      <c r="A110" s="22" t="n">
         <v>45803</v>
       </c>
       <c r="B110" s="14" t="inlineStr">
@@ -5464,7 +5465,7 @@
       <c r="N110" s="17" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="13" t="n">
+      <c r="A111" s="22" t="n">
         <v>45804</v>
       </c>
       <c r="B111" s="14" t="inlineStr">
@@ -5514,7 +5515,7 @@
       <c r="N111" s="17" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="13" t="n">
+      <c r="A112" s="22" t="n">
         <v>45805</v>
       </c>
       <c r="B112" s="14" t="inlineStr">
@@ -5554,7 +5555,7 @@
       <c r="N112" s="17" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="13" t="n">
+      <c r="A113" s="22" t="n">
         <v>45806</v>
       </c>
       <c r="B113" s="14" t="inlineStr">
@@ -5594,7 +5595,7 @@
       <c r="N113" s="17" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="13" t="n">
+      <c r="A114" s="22" t="n">
         <v>45807</v>
       </c>
       <c r="B114" s="14" t="inlineStr">
@@ -5644,7 +5645,7 @@
       <c r="N114" s="17" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="13" t="n">
+      <c r="A115" s="22" t="n">
         <v>45810</v>
       </c>
       <c r="B115" s="14" t="inlineStr">
@@ -5694,7 +5695,7 @@
       <c r="N115" s="17" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="13" t="n">
+      <c r="A116" s="22" t="n">
         <v>45811</v>
       </c>
       <c r="B116" s="14" t="inlineStr">
@@ -5744,7 +5745,7 @@
       <c r="N116" s="17" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="13" t="n">
+      <c r="A117" s="22" t="n">
         <v>45812</v>
       </c>
       <c r="B117" s="14" t="inlineStr">
@@ -5794,7 +5795,7 @@
       <c r="N117" s="17" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="13" t="n">
+      <c r="A118" s="22" t="n">
         <v>45813</v>
       </c>
       <c r="B118" s="14" t="inlineStr">
@@ -5844,7 +5845,7 @@
       <c r="N118" s="17" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="13" t="n">
+      <c r="A119" s="22" t="n">
         <v>45814</v>
       </c>
       <c r="B119" s="14" t="inlineStr">
@@ -5884,7 +5885,7 @@
       <c r="N119" s="17" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="13" t="n">
+      <c r="A120" s="22" t="n">
         <v>45817</v>
       </c>
       <c r="B120" s="14" t="inlineStr">
@@ -5934,7 +5935,7 @@
       <c r="N120" s="17" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="13" t="n">
+      <c r="A121" s="22" t="n">
         <v>45818</v>
       </c>
       <c r="B121" s="14" t="inlineStr">
@@ -5984,7 +5985,7 @@
       <c r="N121" s="17" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="13" t="n">
+      <c r="A122" s="22" t="n">
         <v>45819</v>
       </c>
       <c r="B122" s="14" t="inlineStr">
@@ -6034,7 +6035,7 @@
       <c r="N122" s="17" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="13" t="n">
+      <c r="A123" s="22" t="n">
         <v>45820</v>
       </c>
       <c r="B123" s="14" t="inlineStr">
@@ -6084,7 +6085,7 @@
       <c r="N123" s="17" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="13" t="n">
+      <c r="A124" s="22" t="n">
         <v>45821</v>
       </c>
       <c r="B124" s="14" t="inlineStr">
@@ -6124,7 +6125,7 @@
       <c r="N124" s="17" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="13" t="n">
+      <c r="A125" s="22" t="n">
         <v>45824</v>
       </c>
       <c r="B125" s="14" t="inlineStr">
@@ -6174,7 +6175,7 @@
       <c r="N125" s="17" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="13" t="n">
+      <c r="A126" s="22" t="n">
         <v>45825</v>
       </c>
       <c r="B126" s="14" t="inlineStr">
@@ -6214,7 +6215,7 @@
       <c r="N126" s="17" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="13" t="n">
+      <c r="A127" s="22" t="n">
         <v>45826</v>
       </c>
       <c r="B127" s="14" t="inlineStr">
@@ -6264,7 +6265,7 @@
       <c r="N127" s="17" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="13" t="n">
+      <c r="A128" s="22" t="n">
         <v>45827</v>
       </c>
       <c r="B128" s="14" t="inlineStr">
@@ -6314,7 +6315,7 @@
       <c r="N128" s="17" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="13" t="n">
+      <c r="A129" s="22" t="n">
         <v>45828</v>
       </c>
       <c r="B129" s="14" t="inlineStr">
@@ -6364,7 +6365,7 @@
       <c r="N129" s="17" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="13" t="n">
+      <c r="A130" s="22" t="n">
         <v>45831</v>
       </c>
       <c r="B130" s="14" t="inlineStr">
@@ -6414,7 +6415,7 @@
       <c r="N130" s="17" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="13" t="n">
+      <c r="A131" s="22" t="n">
         <v>45832</v>
       </c>
       <c r="B131" s="14" t="inlineStr">
@@ -6464,7 +6465,7 @@
       <c r="N131" s="17" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="13" t="n">
+      <c r="A132" s="22" t="n">
         <v>45833</v>
       </c>
       <c r="B132" s="14" t="inlineStr">
@@ -6514,7 +6515,7 @@
       <c r="N132" s="17" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="13" t="n">
+      <c r="A133" s="22" t="n">
         <v>45834</v>
       </c>
       <c r="B133" s="14" t="inlineStr">
@@ -6554,7 +6555,7 @@
       <c r="N133" s="17" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="13" t="n">
+      <c r="A134" s="22" t="n">
         <v>45835</v>
       </c>
       <c r="B134" s="14" t="inlineStr">
@@ -6604,7 +6605,7 @@
       <c r="N134" s="17" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="13" t="n">
+      <c r="A135" s="22" t="n">
         <v>45838</v>
       </c>
       <c r="B135" s="14" t="inlineStr">
@@ -6654,7 +6655,7 @@
       <c r="N135" s="17" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="13" t="n">
+      <c r="A136" s="22" t="n">
         <v>45839</v>
       </c>
       <c r="B136" s="14" t="inlineStr">
@@ -6704,7 +6705,7 @@
       <c r="N136" s="17" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="13" t="n">
+      <c r="A137" s="22" t="n">
         <v>45840</v>
       </c>
       <c r="B137" s="14" t="inlineStr">
@@ -6744,7 +6745,7 @@
       <c r="N137" s="17" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="13" t="n">
+      <c r="A138" s="22" t="n">
         <v>45841</v>
       </c>
       <c r="B138" s="14" t="inlineStr">
@@ -6784,7 +6785,7 @@
       <c r="N138" s="17" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="13" t="n">
+      <c r="A139" s="22" t="n">
         <v>45842</v>
       </c>
       <c r="B139" s="14" t="inlineStr">
@@ -6834,7 +6835,7 @@
       <c r="N139" s="17" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="13" t="n">
+      <c r="A140" s="22" t="n">
         <v>45845</v>
       </c>
       <c r="B140" s="14" t="inlineStr">
@@ -6884,7 +6885,7 @@
       <c r="N140" s="17" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="13" t="n">
+      <c r="A141" s="22" t="n">
         <v>45846</v>
       </c>
       <c r="B141" s="14" t="inlineStr">
@@ -6924,7 +6925,7 @@
       <c r="N141" s="17" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="13" t="n">
+      <c r="A142" s="22" t="n">
         <v>45847</v>
       </c>
       <c r="B142" s="14" t="inlineStr">
@@ -6964,7 +6965,7 @@
       <c r="N142" s="17" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="13" t="n">
+      <c r="A143" s="22" t="n">
         <v>45848</v>
       </c>
       <c r="B143" s="14" t="inlineStr">
@@ -6994,7 +6995,7 @@
       <c r="N143" s="17" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="13" t="n">
+      <c r="A144" s="22" t="n">
         <v>45849</v>
       </c>
       <c r="B144" s="14" t="inlineStr">
@@ -7034,7 +7035,7 @@
       <c r="N144" s="17" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="13" t="n">
+      <c r="A145" s="22" t="n">
         <v>45852</v>
       </c>
       <c r="B145" s="14" t="inlineStr">
@@ -7064,7 +7065,7 @@
       <c r="N145" s="17" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="13" t="n">
+      <c r="A146" s="22" t="n">
         <v>45853</v>
       </c>
       <c r="B146" s="14" t="inlineStr">
@@ -7114,7 +7115,7 @@
       <c r="N146" s="17" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="13" t="n">
+      <c r="A147" s="22" t="n">
         <v>45854</v>
       </c>
       <c r="B147" s="14" t="inlineStr">
@@ -7164,7 +7165,7 @@
       <c r="N147" s="17" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="13" t="n">
+      <c r="A148" s="22" t="n">
         <v>45855</v>
       </c>
       <c r="B148" s="14" t="inlineStr">
@@ -7214,7 +7215,7 @@
       <c r="N148" s="17" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="13" t="n">
+      <c r="A149" s="22" t="n">
         <v>45856</v>
       </c>
       <c r="B149" s="14" t="inlineStr">
@@ -7254,7 +7255,7 @@
       <c r="N149" s="17" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="13" t="n">
+      <c r="A150" s="22" t="n">
         <v>45859</v>
       </c>
       <c r="B150" s="14" t="inlineStr">
@@ -7304,7 +7305,7 @@
       <c r="N150" s="17" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="13" t="n">
+      <c r="A151" s="22" t="n">
         <v>45860</v>
       </c>
       <c r="B151" s="14" t="inlineStr">
@@ -7354,7 +7355,7 @@
       <c r="N151" s="17" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="13" t="n">
+      <c r="A152" s="22" t="n">
         <v>45861</v>
       </c>
       <c r="B152" s="14" t="inlineStr">
@@ -7404,7 +7405,7 @@
       <c r="N152" s="17" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="13" t="n">
+      <c r="A153" s="22" t="n">
         <v>45862</v>
       </c>
       <c r="B153" s="14" t="inlineStr">
@@ -7454,7 +7455,7 @@
       <c r="N153" s="17" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="13" t="n">
+      <c r="A154" s="22" t="n">
         <v>45863</v>
       </c>
       <c r="B154" s="14" t="inlineStr">
@@ -7504,7 +7505,7 @@
       <c r="N154" s="17" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="13" t="n">
+      <c r="A155" s="22" t="n">
         <v>45866</v>
       </c>
       <c r="B155" s="14" t="inlineStr">
@@ -7544,7 +7545,7 @@
       <c r="N155" s="17" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="13" t="n">
+      <c r="A156" s="22" t="n">
         <v>45867</v>
       </c>
       <c r="B156" s="14" t="inlineStr">
@@ -7594,7 +7595,7 @@
       <c r="N156" s="17" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="13" t="n">
+      <c r="A157" s="22" t="n">
         <v>45868</v>
       </c>
       <c r="B157" s="14" t="inlineStr">
@@ -7634,7 +7635,7 @@
       <c r="N157" s="17" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="13" t="n">
+      <c r="A158" s="22" t="n">
         <v>45869</v>
       </c>
       <c r="B158" s="14" t="inlineStr">
@@ -7684,7 +7685,7 @@
       <c r="N158" s="17" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="13" t="n">
+      <c r="A159" s="22" t="n">
         <v>45870</v>
       </c>
       <c r="B159" s="14" t="inlineStr">
@@ -7734,7 +7735,7 @@
       <c r="N159" s="17" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="13" t="n">
+      <c r="A160" s="22" t="n">
         <v>45873</v>
       </c>
       <c r="B160" s="14" t="inlineStr">
@@ -7784,7 +7785,7 @@
       <c r="N160" s="17" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" s="13" t="n">
+      <c r="A161" s="22" t="n">
         <v>45874</v>
       </c>
       <c r="B161" s="14" t="inlineStr">
@@ -7824,7 +7825,7 @@
       <c r="N161" s="17" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="13" t="n">
+      <c r="A162" s="22" t="n">
         <v>45875</v>
       </c>
       <c r="B162" s="14" t="inlineStr">
@@ -7854,7 +7855,7 @@
       <c r="N162" s="17" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" s="13" t="n">
+      <c r="A163" s="22" t="n">
         <v>45876</v>
       </c>
       <c r="B163" s="14" t="inlineStr">
@@ -7894,7 +7895,7 @@
       <c r="N163" s="17" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" s="13" t="n">
+      <c r="A164" s="22" t="n">
         <v>45877</v>
       </c>
       <c r="B164" s="14" t="inlineStr">
@@ -7934,7 +7935,7 @@
       <c r="N164" s="17" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="13" t="n">
+      <c r="A165" s="22" t="n">
         <v>45880</v>
       </c>
       <c r="B165" s="14" t="inlineStr">
@@ -7964,7 +7965,7 @@
       <c r="N165" s="17" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" s="13" t="n">
+      <c r="A166" s="22" t="n">
         <v>45881</v>
       </c>
       <c r="B166" s="14" t="inlineStr">
@@ -8014,7 +8015,7 @@
       <c r="N166" s="17" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" s="13" t="n">
+      <c r="A167" s="22" t="n">
         <v>45882</v>
       </c>
       <c r="B167" s="14" t="inlineStr">
@@ -8054,7 +8055,7 @@
       <c r="N167" s="17" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="13" t="n">
+      <c r="A168" s="22" t="n">
         <v>45883</v>
       </c>
       <c r="B168" s="14" t="inlineStr">
@@ -8104,7 +8105,7 @@
       <c r="N168" s="17" t="n"/>
     </row>
     <row r="169">
-      <c r="A169" s="13" t="n">
+      <c r="A169" s="22" t="n">
         <v>45884</v>
       </c>
       <c r="B169" s="14" t="inlineStr">
@@ -8144,7 +8145,7 @@
       <c r="N169" s="17" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" s="13" t="n">
+      <c r="A170" s="22" t="n">
         <v>45887</v>
       </c>
       <c r="B170" s="14" t="inlineStr">
@@ -8194,7 +8195,7 @@
       <c r="N170" s="17" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" s="13" t="n">
+      <c r="A171" s="22" t="n">
         <v>45888</v>
       </c>
       <c r="B171" s="14" t="inlineStr">
@@ -8234,7 +8235,7 @@
       <c r="N171" s="17" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="13" t="n">
+      <c r="A172" s="22" t="n">
         <v>45889</v>
       </c>
       <c r="B172" s="14" t="inlineStr">
@@ -8274,7 +8275,7 @@
       <c r="N172" s="17" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" s="13" t="n">
+      <c r="A173" s="22" t="n">
         <v>45890</v>
       </c>
       <c r="B173" s="14" t="inlineStr">
@@ -8324,7 +8325,7 @@
       <c r="N173" s="17" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" s="13" t="n">
+      <c r="A174" s="22" t="n">
         <v>45891</v>
       </c>
       <c r="B174" s="14" t="inlineStr">
@@ -8374,7 +8375,7 @@
       <c r="N174" s="17" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="13" t="n">
+      <c r="A175" s="22" t="n">
         <v>45894</v>
       </c>
       <c r="B175" s="14" t="inlineStr">
@@ -8414,7 +8415,7 @@
       <c r="N175" s="17" t="n"/>
     </row>
     <row r="176">
-      <c r="A176" s="13" t="n">
+      <c r="A176" s="22" t="n">
         <v>45895</v>
       </c>
       <c r="B176" s="14" t="inlineStr">
@@ -8454,7 +8455,7 @@
       <c r="N176" s="17" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" s="13" t="n">
+      <c r="A177" s="22" t="n">
         <v>45896</v>
       </c>
       <c r="B177" s="14" t="inlineStr">
@@ -8494,7 +8495,7 @@
       <c r="N177" s="17" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" s="13" t="n">
+      <c r="A178" s="22" t="n">
         <v>45897</v>
       </c>
       <c r="B178" s="14" t="inlineStr">
@@ -8544,7 +8545,7 @@
       <c r="N178" s="17" t="n"/>
     </row>
     <row r="179">
-      <c r="A179" s="13" t="n">
+      <c r="A179" s="22" t="n">
         <v>45898</v>
       </c>
       <c r="B179" s="14" t="inlineStr">
@@ -8594,7 +8595,7 @@
       <c r="N179" s="17" t="n"/>
     </row>
     <row r="180">
-      <c r="A180" s="13" t="n">
+      <c r="A180" s="22" t="n">
         <v>45901</v>
       </c>
       <c r="B180" s="14" t="inlineStr">
@@ -8634,7 +8635,7 @@
       <c r="N180" s="17" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" s="13" t="n">
+      <c r="A181" s="22" t="n">
         <v>45902</v>
       </c>
       <c r="B181" s="14" t="inlineStr">
@@ -8684,7 +8685,7 @@
       <c r="N181" s="17" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="13" t="n">
+      <c r="A182" s="22" t="n">
         <v>45903</v>
       </c>
       <c r="B182" s="14" t="inlineStr">
@@ -8734,7 +8735,7 @@
       <c r="N182" s="17" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="13" t="n">
+      <c r="A183" s="22" t="n">
         <v>45904</v>
       </c>
       <c r="B183" s="14" t="inlineStr">
@@ -8784,7 +8785,7 @@
       <c r="N183" s="17" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="13" t="n">
+      <c r="A184" s="22" t="n">
         <v>45905</v>
       </c>
       <c r="B184" s="14" t="inlineStr">
@@ -8824,7 +8825,7 @@
       <c r="N184" s="17" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" s="13" t="n">
+      <c r="A185" s="22" t="n">
         <v>45908</v>
       </c>
       <c r="B185" s="14" t="inlineStr">
@@ -8874,7 +8875,7 @@
       <c r="N185" s="17" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="13" t="n">
+      <c r="A186" s="22" t="n">
         <v>45909</v>
       </c>
       <c r="B186" s="14" t="inlineStr">
@@ -8924,7 +8925,7 @@
       <c r="N186" s="17" t="n"/>
     </row>
     <row r="187">
-      <c r="A187" s="13" t="n">
+      <c r="A187" s="22" t="n">
         <v>45910</v>
       </c>
       <c r="B187" s="14" t="inlineStr">
@@ -8974,7 +8975,7 @@
       <c r="N187" s="17" t="n"/>
     </row>
     <row r="188">
-      <c r="A188" s="13" t="n">
+      <c r="A188" s="22" t="n">
         <v>45911</v>
       </c>
       <c r="B188" s="14" t="inlineStr">
@@ -9024,7 +9025,7 @@
       <c r="N188" s="17" t="n"/>
     </row>
     <row r="189">
-      <c r="A189" s="13" t="n">
+      <c r="A189" s="22" t="n">
         <v>45912</v>
       </c>
       <c r="B189" s="14" t="inlineStr">
@@ -9074,7 +9075,7 @@
       <c r="N189" s="17" t="n"/>
     </row>
     <row r="190">
-      <c r="A190" s="13" t="n">
+      <c r="A190" s="22" t="n">
         <v>45915</v>
       </c>
       <c r="B190" s="14" t="inlineStr">
@@ -9124,7 +9125,7 @@
       <c r="N190" s="17" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="13" t="n">
+      <c r="A191" s="22" t="n">
         <v>45916</v>
       </c>
       <c r="B191" s="14" t="inlineStr">
@@ -9164,7 +9165,7 @@
       <c r="N191" s="17" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="13" t="n">
+      <c r="A192" s="22" t="n">
         <v>45917</v>
       </c>
       <c r="B192" s="14" t="inlineStr">
@@ -9204,7 +9205,7 @@
       <c r="N192" s="17" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="13" t="n">
+      <c r="A193" s="22" t="n">
         <v>45918</v>
       </c>
       <c r="B193" s="14" t="inlineStr">
@@ -9254,7 +9255,7 @@
       <c r="N193" s="17" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="13" t="n">
+      <c r="A194" s="22" t="n">
         <v>45919</v>
       </c>
       <c r="B194" s="14" t="inlineStr">
@@ -9304,7 +9305,7 @@
       <c r="N194" s="17" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="13" t="n">
+      <c r="A195" s="22" t="n">
         <v>45922</v>
       </c>
       <c r="B195" s="14" t="inlineStr">
@@ -9354,7 +9355,7 @@
       <c r="N195" s="17" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="13" t="n">
+      <c r="A196" s="22" t="n">
         <v>45923</v>
       </c>
       <c r="B196" s="14" t="inlineStr">
@@ -9404,7 +9405,7 @@
       <c r="N196" s="17" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="13" t="n">
+      <c r="A197" s="22" t="n">
         <v>45924</v>
       </c>
       <c r="B197" s="14" t="inlineStr">
@@ -9444,7 +9445,7 @@
       <c r="N197" s="17" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="13" t="n">
+      <c r="A198" s="22" t="n">
         <v>45925</v>
       </c>
       <c r="B198" s="14" t="inlineStr">
@@ -9494,7 +9495,7 @@
       <c r="N198" s="17" t="n"/>
     </row>
     <row r="199">
-      <c r="A199" s="13" t="n">
+      <c r="A199" s="22" t="n">
         <v>45926</v>
       </c>
       <c r="B199" s="14" t="inlineStr">
@@ -9544,7 +9545,7 @@
       <c r="N199" s="17" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" s="13" t="n">
+      <c r="A200" s="22" t="n">
         <v>45929</v>
       </c>
       <c r="B200" s="14" t="inlineStr">
@@ -9594,7 +9595,7 @@
       <c r="N200" s="17" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" s="13" t="n">
+      <c r="A201" s="22" t="n">
         <v>45930</v>
       </c>
       <c r="B201" s="14" t="inlineStr">
@@ -9634,7 +9635,7 @@
       <c r="N201" s="17" t="n"/>
     </row>
     <row r="202">
-      <c r="A202" s="13" t="n">
+      <c r="A202" s="22" t="n">
         <v>45931</v>
       </c>
       <c r="B202" s="14" t="inlineStr">
@@ -9684,7 +9685,7 @@
       <c r="N202" s="17" t="n"/>
     </row>
     <row r="203">
-      <c r="A203" s="13" t="n">
+      <c r="A203" s="22" t="n">
         <v>45932</v>
       </c>
       <c r="B203" s="14" t="inlineStr">
@@ -9734,7 +9735,7 @@
       <c r="N203" s="17" t="n"/>
     </row>
     <row r="204">
-      <c r="A204" s="13" t="n">
+      <c r="A204" s="22" t="n">
         <v>45933</v>
       </c>
       <c r="B204" s="14" t="inlineStr">
@@ -9774,7 +9775,7 @@
       <c r="N204" s="17" t="n"/>
     </row>
     <row r="205">
-      <c r="A205" s="13" t="n">
+      <c r="A205" s="22" t="n">
         <v>45936</v>
       </c>
       <c r="B205" s="14" t="inlineStr">
@@ -9824,7 +9825,7 @@
       <c r="N205" s="17" t="n"/>
     </row>
     <row r="206">
-      <c r="A206" s="13" t="n">
+      <c r="A206" s="22" t="n">
         <v>45937</v>
       </c>
       <c r="B206" s="14" t="inlineStr">
@@ -9864,7 +9865,7 @@
       <c r="N206" s="17" t="n"/>
     </row>
     <row r="207">
-      <c r="A207" s="13" t="n">
+      <c r="A207" s="22" t="n">
         <v>45938</v>
       </c>
       <c r="B207" s="14" t="inlineStr">
@@ -9914,7 +9915,7 @@
       <c r="N207" s="17" t="n"/>
     </row>
     <row r="208">
-      <c r="A208" s="13" t="n">
+      <c r="A208" s="22" t="n">
         <v>45939</v>
       </c>
       <c r="B208" s="14" t="inlineStr">
@@ -9964,7 +9965,7 @@
       <c r="N208" s="17" t="n"/>
     </row>
     <row r="209">
-      <c r="A209" s="13" t="n">
+      <c r="A209" s="22" t="n">
         <v>45940</v>
       </c>
       <c r="B209" s="14" t="inlineStr">
@@ -10014,7 +10015,7 @@
       <c r="N209" s="17" t="n"/>
     </row>
     <row r="210">
-      <c r="A210" s="13" t="n">
+      <c r="A210" s="22" t="n">
         <v>45943</v>
       </c>
       <c r="B210" s="14" t="inlineStr">
@@ -10064,7 +10065,7 @@
       <c r="N210" s="17" t="n"/>
     </row>
     <row r="211">
-      <c r="A211" s="13" t="n">
+      <c r="A211" s="22" t="n">
         <v>45944</v>
       </c>
       <c r="B211" s="14" t="inlineStr">
@@ -10104,7 +10105,7 @@
       <c r="N211" s="17" t="n"/>
     </row>
     <row r="212">
-      <c r="A212" s="13" t="n">
+      <c r="A212" s="22" t="n">
         <v>45945</v>
       </c>
       <c r="B212" s="14" t="inlineStr">
@@ -10154,7 +10155,7 @@
       <c r="N212" s="17" t="n"/>
     </row>
     <row r="213">
-      <c r="A213" s="13" t="n">
+      <c r="A213" s="22" t="n">
         <v>45946</v>
       </c>
       <c r="B213" s="14" t="inlineStr">
@@ -10184,7 +10185,7 @@
       <c r="N213" s="17" t="n"/>
     </row>
     <row r="214">
-      <c r="A214" s="13" t="n">
+      <c r="A214" s="22" t="n">
         <v>45947</v>
       </c>
       <c r="B214" s="14" t="inlineStr">
@@ -10234,7 +10235,7 @@
       <c r="N214" s="17" t="n"/>
     </row>
     <row r="215">
-      <c r="A215" s="13" t="n">
+      <c r="A215" s="22" t="n">
         <v>45950</v>
       </c>
       <c r="B215" s="14" t="inlineStr">
@@ -10284,7 +10285,7 @@
       <c r="N215" s="17" t="n"/>
     </row>
     <row r="216">
-      <c r="A216" s="13" t="n">
+      <c r="A216" s="22" t="n">
         <v>45951</v>
       </c>
       <c r="B216" s="14" t="inlineStr">
@@ -10334,7 +10335,7 @@
       <c r="N216" s="17" t="n"/>
     </row>
     <row r="217">
-      <c r="A217" s="13" t="n">
+      <c r="A217" s="22" t="n">
         <v>45952</v>
       </c>
       <c r="B217" s="14" t="inlineStr">
@@ -10384,7 +10385,7 @@
       <c r="N217" s="17" t="n"/>
     </row>
     <row r="218">
-      <c r="A218" s="13" t="n">
+      <c r="A218" s="22" t="n">
         <v>45953</v>
       </c>
       <c r="B218" s="14" t="inlineStr">
@@ -10424,7 +10425,7 @@
       <c r="N218" s="17" t="n"/>
     </row>
     <row r="219">
-      <c r="A219" s="13" t="n">
+      <c r="A219" s="22" t="n">
         <v>45954</v>
       </c>
       <c r="B219" s="14" t="inlineStr">
@@ -10474,7 +10475,7 @@
       <c r="N219" s="17" t="n"/>
     </row>
     <row r="220">
-      <c r="A220" s="13" t="n">
+      <c r="A220" s="22" t="n">
         <v>45957</v>
       </c>
       <c r="B220" s="14" t="inlineStr">
@@ -10524,7 +10525,7 @@
       <c r="N220" s="17" t="n"/>
     </row>
     <row r="221">
-      <c r="A221" s="13" t="n">
+      <c r="A221" s="22" t="n">
         <v>45958</v>
       </c>
       <c r="B221" s="14" t="inlineStr">
@@ -10574,7 +10575,7 @@
       <c r="N221" s="17" t="n"/>
     </row>
     <row r="222">
-      <c r="A222" s="13" t="n">
+      <c r="A222" s="22" t="n">
         <v>45959</v>
       </c>
       <c r="B222" s="14" t="inlineStr">
@@ -10624,7 +10625,7 @@
       <c r="N222" s="17" t="n"/>
     </row>
     <row r="223">
-      <c r="A223" s="13" t="n">
+      <c r="A223" s="22" t="n">
         <v>45960</v>
       </c>
       <c r="B223" s="14" t="inlineStr">
@@ -10664,7 +10665,7 @@
       <c r="N223" s="17" t="n"/>
     </row>
     <row r="224">
-      <c r="A224" s="13" t="n">
+      <c r="A224" s="22" t="n">
         <v>45961</v>
       </c>
       <c r="B224" s="14" t="inlineStr">
@@ -10704,7 +10705,7 @@
       <c r="N224" s="17" t="n"/>
     </row>
     <row r="225">
-      <c r="A225" s="13" t="n">
+      <c r="A225" s="22" t="n">
         <v>45964</v>
       </c>
       <c r="B225" s="14" t="inlineStr">
@@ -10754,7 +10755,7 @@
       <c r="N225" s="17" t="n"/>
     </row>
     <row r="226">
-      <c r="A226" s="13" t="n">
+      <c r="A226" s="22" t="n">
         <v>45965</v>
       </c>
       <c r="B226" s="14" t="inlineStr">
@@ -10804,7 +10805,7 @@
       <c r="N226" s="17" t="n"/>
     </row>
     <row r="227">
-      <c r="A227" s="13" t="n">
+      <c r="A227" s="22" t="n">
         <v>45966</v>
       </c>
       <c r="B227" s="14" t="inlineStr">
@@ -10844,7 +10845,7 @@
       <c r="N227" s="17" t="n"/>
     </row>
     <row r="228">
-      <c r="A228" s="13" t="n">
+      <c r="A228" s="22" t="n">
         <v>45967</v>
       </c>
       <c r="B228" s="14" t="inlineStr">
@@ -10894,7 +10895,7 @@
       <c r="N228" s="17" t="n"/>
     </row>
     <row r="229">
-      <c r="A229" s="13" t="n">
+      <c r="A229" s="22" t="n">
         <v>45968</v>
       </c>
       <c r="B229" s="14" t="inlineStr">
@@ -10944,7 +10945,7 @@
       <c r="N229" s="17" t="n"/>
     </row>
     <row r="230">
-      <c r="A230" s="13" t="n">
+      <c r="A230" s="22" t="n">
         <v>45971</v>
       </c>
       <c r="B230" s="14" t="inlineStr">
@@ -10994,7 +10995,7 @@
       <c r="N230" s="17" t="n"/>
     </row>
     <row r="231">
-      <c r="A231" s="13" t="n">
+      <c r="A231" s="22" t="n">
         <v>45972</v>
       </c>
       <c r="B231" s="14" t="inlineStr">
@@ -11034,7 +11035,7 @@
       <c r="N231" s="17" t="n"/>
     </row>
     <row r="232">
-      <c r="A232" s="13" t="n">
+      <c r="A232" s="22" t="n">
         <v>45973</v>
       </c>
       <c r="B232" s="14" t="inlineStr">
@@ -11084,7 +11085,7 @@
       <c r="N232" s="17" t="n"/>
     </row>
     <row r="233">
-      <c r="A233" s="13" t="n">
+      <c r="A233" s="22" t="n">
         <v>45974</v>
       </c>
       <c r="B233" s="14" t="inlineStr">
@@ -11134,7 +11135,7 @@
       <c r="N233" s="17" t="n"/>
     </row>
     <row r="234">
-      <c r="A234" s="13" t="n">
+      <c r="A234" s="22" t="n">
         <v>45975</v>
       </c>
       <c r="B234" s="14" t="inlineStr">
@@ -11184,7 +11185,7 @@
       <c r="N234" s="17" t="n"/>
     </row>
     <row r="235">
-      <c r="A235" s="13" t="n">
+      <c r="A235" s="22" t="n">
         <v>45978</v>
       </c>
       <c r="B235" s="14" t="inlineStr">
@@ -11224,7 +11225,7 @@
       <c r="N235" s="17" t="n"/>
     </row>
     <row r="236">
-      <c r="A236" s="13" t="n">
+      <c r="A236" s="22" t="n">
         <v>45979</v>
       </c>
       <c r="B236" s="14" t="inlineStr">
@@ -11274,7 +11275,7 @@
       <c r="N236" s="17" t="n"/>
     </row>
     <row r="237">
-      <c r="A237" s="13" t="n">
+      <c r="A237" s="22" t="n">
         <v>45980</v>
       </c>
       <c r="B237" s="14" t="inlineStr">
@@ -11324,7 +11325,7 @@
       <c r="N237" s="17" t="n"/>
     </row>
     <row r="238">
-      <c r="A238" s="13" t="n">
+      <c r="A238" s="22" t="n">
         <v>45981</v>
       </c>
       <c r="B238" s="14" t="inlineStr">
@@ -11364,7 +11365,7 @@
       <c r="N238" s="17" t="n"/>
     </row>
     <row r="239">
-      <c r="A239" s="13" t="n">
+      <c r="A239" s="22" t="n">
         <v>45982</v>
       </c>
       <c r="B239" s="14" t="inlineStr">
@@ -11414,7 +11415,7 @@
       <c r="N239" s="17" t="n"/>
     </row>
     <row r="240">
-      <c r="A240" s="13" t="n">
+      <c r="A240" s="22" t="n">
         <v>45985</v>
       </c>
       <c r="B240" s="14" t="inlineStr">
@@ -11454,7 +11455,7 @@
       <c r="N240" s="17" t="n"/>
     </row>
     <row r="241">
-      <c r="A241" s="13" t="n">
+      <c r="A241" s="22" t="n">
         <v>45986</v>
       </c>
       <c r="B241" s="14" t="inlineStr">
@@ -11494,7 +11495,7 @@
       <c r="N241" s="17" t="n"/>
     </row>
     <row r="242">
-      <c r="A242" s="13" t="n">
+      <c r="A242" s="22" t="n">
         <v>45987</v>
       </c>
       <c r="B242" s="14" t="inlineStr">
@@ -11544,7 +11545,7 @@
       <c r="N242" s="17" t="n"/>
     </row>
     <row r="243">
-      <c r="A243" s="13" t="n">
+      <c r="A243" s="22" t="n">
         <v>45988</v>
       </c>
       <c r="B243" s="14" t="inlineStr">
@@ -11594,7 +11595,7 @@
       <c r="N243" s="17" t="n"/>
     </row>
     <row r="244">
-      <c r="A244" s="13" t="n">
+      <c r="A244" s="22" t="n">
         <v>45989</v>
       </c>
       <c r="B244" s="14" t="inlineStr">
@@ -11634,7 +11635,7 @@
       <c r="N244" s="17" t="n"/>
     </row>
     <row r="245">
-      <c r="A245" s="13" t="n">
+      <c r="A245" s="22" t="n">
         <v>45992</v>
       </c>
       <c r="B245" s="14" t="inlineStr">
@@ -11684,7 +11685,7 @@
       <c r="N245" s="17" t="n"/>
     </row>
     <row r="246">
-      <c r="A246" s="13" t="n">
+      <c r="A246" s="22" t="n">
         <v>45993</v>
       </c>
       <c r="B246" s="14" t="inlineStr">
@@ -11734,7 +11735,7 @@
       <c r="N246" s="17" t="n"/>
     </row>
     <row r="247">
-      <c r="A247" s="13" t="n">
+      <c r="A247" s="22" t="n">
         <v>45994</v>
       </c>
       <c r="B247" s="14" t="inlineStr">
@@ -11784,7 +11785,7 @@
       <c r="N247" s="17" t="n"/>
     </row>
     <row r="248">
-      <c r="A248" s="13" t="n">
+      <c r="A248" s="22" t="n">
         <v>45995</v>
       </c>
       <c r="B248" s="14" t="inlineStr">
@@ -11834,7 +11835,7 @@
       <c r="N248" s="17" t="n"/>
     </row>
     <row r="249">
-      <c r="A249" s="13" t="n">
+      <c r="A249" s="22" t="n">
         <v>45996</v>
       </c>
       <c r="B249" s="14" t="inlineStr">
@@ -11884,7 +11885,7 @@
       <c r="N249" s="17" t="n"/>
     </row>
     <row r="250">
-      <c r="A250" s="13" t="n">
+      <c r="A250" s="22" t="n">
         <v>45999</v>
       </c>
       <c r="B250" s="14" t="inlineStr">
@@ -11934,7 +11935,7 @@
       <c r="N250" s="17" t="n"/>
     </row>
     <row r="251">
-      <c r="A251" s="13" t="n">
+      <c r="A251" s="22" t="n">
         <v>46000</v>
       </c>
       <c r="B251" s="14" t="inlineStr">
@@ -11984,7 +11985,7 @@
       <c r="N251" s="17" t="n"/>
     </row>
     <row r="252">
-      <c r="A252" s="13" t="n">
+      <c r="A252" s="22" t="n">
         <v>46001</v>
       </c>
       <c r="B252" s="14" t="inlineStr">
@@ -12034,7 +12035,7 @@
       <c r="N252" s="17" t="n"/>
     </row>
     <row r="253">
-      <c r="A253" s="13" t="n">
+      <c r="A253" s="22" t="n">
         <v>46002</v>
       </c>
       <c r="B253" s="14" t="inlineStr">
@@ -12074,7 +12075,7 @@
       <c r="N253" s="17" t="n"/>
     </row>
     <row r="254">
-      <c r="A254" s="13" t="n">
+      <c r="A254" s="22" t="n">
         <v>46003</v>
       </c>
       <c r="B254" s="14" t="inlineStr">
@@ -12124,7 +12125,7 @@
       <c r="N254" s="17" t="n"/>
     </row>
     <row r="255">
-      <c r="A255" s="13" t="n">
+      <c r="A255" s="22" t="n">
         <v>46006</v>
       </c>
       <c r="B255" s="14" t="inlineStr">
@@ -12174,7 +12175,7 @@
       <c r="N255" s="17" t="n"/>
     </row>
     <row r="256">
-      <c r="A256" s="13" t="n">
+      <c r="A256" s="22" t="n">
         <v>46007</v>
       </c>
       <c r="B256" s="14" t="inlineStr">
@@ -12224,7 +12225,7 @@
       <c r="N256" s="17" t="n"/>
     </row>
     <row r="257">
-      <c r="A257" s="13" t="n">
+      <c r="A257" s="22" t="n">
         <v>46008</v>
       </c>
       <c r="B257" s="14" t="inlineStr">
@@ -12274,7 +12275,7 @@
       <c r="N257" s="17" t="n"/>
     </row>
     <row r="258">
-      <c r="A258" s="13" t="n">
+      <c r="A258" s="22" t="n">
         <v>46009</v>
       </c>
       <c r="B258" s="14" t="inlineStr">
@@ -12324,7 +12325,7 @@
       <c r="N258" s="17" t="n"/>
     </row>
     <row r="259">
-      <c r="A259" s="13" t="n">
+      <c r="A259" s="22" t="n">
         <v>46010</v>
       </c>
       <c r="B259" s="14" t="inlineStr">
@@ -12374,7 +12375,7 @@
       <c r="N259" s="17" t="n"/>
     </row>
     <row r="260">
-      <c r="A260" s="13" t="n">
+      <c r="A260" s="22" t="n">
         <v>46013</v>
       </c>
       <c r="B260" s="14" t="inlineStr">
@@ -12414,7 +12415,7 @@
       <c r="N260" s="17" t="n"/>
     </row>
     <row r="261">
-      <c r="A261" s="13" t="n">
+      <c r="A261" s="22" t="n">
         <v>46014</v>
       </c>
       <c r="B261" s="14" t="inlineStr">
@@ -12464,7 +12465,7 @@
       <c r="N261" s="17" t="n"/>
     </row>
     <row r="262">
-      <c r="A262" s="13" t="n">
+      <c r="A262" s="22" t="n">
         <v>46015</v>
       </c>
       <c r="B262" s="14" t="inlineStr">
@@ -12514,7 +12515,7 @@
       <c r="N262" s="17" t="n"/>
     </row>
     <row r="263">
-      <c r="A263" s="11" t="n">
+      <c r="A263" s="21" t="n">
         <v>46016</v>
       </c>
       <c r="B263" s="12" t="inlineStr">
@@ -12544,7 +12545,7 @@
       <c r="N263" s="12" t="n"/>
     </row>
     <row r="264">
-      <c r="A264" s="13" t="n">
+      <c r="A264" s="22" t="n">
         <v>46017</v>
       </c>
       <c r="B264" s="14" t="inlineStr">
@@ -12584,7 +12585,7 @@
       <c r="N264" s="17" t="n"/>
     </row>
     <row r="265">
-      <c r="A265" s="13" t="n">
+      <c r="A265" s="22" t="n">
         <v>46020</v>
       </c>
       <c r="B265" s="14" t="inlineStr">
@@ -12624,7 +12625,7 @@
       <c r="N265" s="17" t="n"/>
     </row>
     <row r="266">
-      <c r="A266" s="13" t="n">
+      <c r="A266" s="22" t="n">
         <v>46021</v>
       </c>
       <c r="B266" s="14" t="inlineStr">
@@ -12674,7 +12675,7 @@
       <c r="N266" s="17" t="n"/>
     </row>
     <row r="267">
-      <c r="A267" s="13" t="n">
+      <c r="A267" s="22" t="n">
         <v>46022</v>
       </c>
       <c r="B267" s="14" t="inlineStr">
@@ -12713,10 +12714,16 @@
       <c r="M267" s="16" t="n"/>
       <c r="N267" s="17" t="n"/>
     </row>
+    <row r="268"/>
     <row r="269">
       <c r="A269" s="19" t="inlineStr">
         <is>
           <t>RESUMEN (automático)</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>(las cifras aparecen al abrir el fichero en Excel o Google Sheets)</t>
         </is>
       </c>
     </row>

</xml_diff>